<commit_message>
test: update BVA and whitebox order payment
</commit_message>
<xml_diff>
--- a/docs/testing/WhiteBox/Oder_Payment/Testcase_Whitebox_Order_Payment.xlsx
+++ b/docs/testing/WhiteBox/Oder_Payment/Testcase_Whitebox_Order_Payment.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000"/>
+    <workbookView windowWidth="15732" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Whitebox_TestCases" sheetId="1" r:id="rId1"/>
@@ -32,13 +32,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="290">
   <si>
-    <t>Test Case ID*</t>
+    <t>Test Case ID</t>
   </si>
   <si>
     <t>Module</t>
   </si>
   <si>
-    <t>Test Summary / Description*</t>
+    <t>Test Summary / Description</t>
   </si>
   <si>
     <t>Kỹ thuật / Tiêu chí White-box (Statement/Branch)</t>
@@ -56,16 +56,16 @@
     <t>Test Steps*</t>
   </si>
   <si>
-    <t>Inputs (Test Data / Request)*</t>
-  </si>
-  <si>
-    <t>Expected Result*</t>
+    <t>Inputs (Test Data / Request)</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
   </si>
   <si>
     <t>Actual Result (Kết quả thực tế)*</t>
   </si>
   <si>
-    <t>Pass/Fail*</t>
+    <t>Pass/Fail</t>
   </si>
   <si>
     <t>TC_WB_01</t>

</xml_diff>